<commit_message>
Dados set/2026 — 57 meses no painel
</commit_message>
<xml_diff>
--- a/dados/excel/genero_evolucao_mensal.xlsx
+++ b/dados/excel/genero_evolucao_mensal.xlsx
@@ -628,7 +628,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>12/10/2026 16:30</t>
+          <t>16/10/2026 19:58</t>
         </is>
       </c>
     </row>
@@ -847,19 +847,19 @@
         <v>1</v>
       </c>
       <c r="C2" s="10" t="n">
-        <v>8603</v>
+        <v>8554</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>151</v>
+        <v>220</v>
       </c>
       <c r="E2" s="10" t="n">
-        <v>2536</v>
+        <v>2516</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>11290</v>
       </c>
       <c r="G2" s="10" t="n">
-        <v>76.2</v>
+        <v>75.77</v>
       </c>
     </row>
     <row r="3">
@@ -870,19 +870,19 @@
         <v>2</v>
       </c>
       <c r="C3" s="13" t="n">
-        <v>7187</v>
+        <v>7149</v>
       </c>
       <c r="D3" s="11" t="n">
-        <v>136</v>
+        <v>193</v>
       </c>
       <c r="E3" s="13" t="n">
-        <v>2406</v>
+        <v>2387</v>
       </c>
       <c r="F3" s="11" t="n">
         <v>9729</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>73.87</v>
+        <v>73.48</v>
       </c>
     </row>
     <row r="4">
@@ -893,19 +893,19 @@
         <v>3</v>
       </c>
       <c r="C4" s="10" t="n">
-        <v>8663</v>
+        <v>8614</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>149</v>
+        <v>218</v>
       </c>
       <c r="E4" s="10" t="n">
-        <v>2525</v>
+        <v>2505</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>11337</v>
       </c>
       <c r="G4" s="10" t="n">
-        <v>76.41</v>
+        <v>75.98</v>
       </c>
     </row>
     <row r="5">
@@ -916,19 +916,19 @@
         <v>4</v>
       </c>
       <c r="C5" s="13" t="n">
-        <v>8901</v>
+        <v>8853</v>
       </c>
       <c r="D5" s="11" t="n">
-        <v>153</v>
+        <v>222</v>
       </c>
       <c r="E5" s="13" t="n">
-        <v>2525</v>
+        <v>2504</v>
       </c>
       <c r="F5" s="11" t="n">
         <v>11579</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>76.87</v>
+        <v>76.45999999999999</v>
       </c>
     </row>
     <row r="6">
@@ -939,19 +939,19 @@
         <v>5</v>
       </c>
       <c r="C6" s="10" t="n">
-        <v>9051</v>
+        <v>9002</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>156</v>
+        <v>226</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>2560</v>
+        <v>2539</v>
       </c>
       <c r="F6" s="8" t="n">
         <v>11767</v>
       </c>
       <c r="G6" s="10" t="n">
-        <v>76.92</v>
+        <v>76.5</v>
       </c>
     </row>
     <row r="7">
@@ -962,19 +962,19 @@
         <v>6</v>
       </c>
       <c r="C7" s="13" t="n">
-        <v>9173</v>
+        <v>9121</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>156</v>
+        <v>230</v>
       </c>
       <c r="E7" s="13" t="n">
-        <v>2586</v>
+        <v>2564</v>
       </c>
       <c r="F7" s="11" t="n">
         <v>11915</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>76.98999999999999</v>
+        <v>76.55</v>
       </c>
     </row>
     <row r="8">
@@ -985,19 +985,19 @@
         <v>7</v>
       </c>
       <c r="C8" s="10" t="n">
-        <v>9066</v>
+        <v>9014</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>153</v>
+        <v>226</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>2574</v>
+        <v>2553</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>11793</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>76.88</v>
+        <v>76.44</v>
       </c>
     </row>
     <row r="9">
@@ -1008,19 +1008,19 @@
         <v>8</v>
       </c>
       <c r="C9" s="13" t="n">
-        <v>9091</v>
+        <v>9042</v>
       </c>
       <c r="D9" s="11" t="n">
-        <v>156</v>
+        <v>227</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>2589</v>
+        <v>2567</v>
       </c>
       <c r="F9" s="11" t="n">
         <v>11836</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>76.81</v>
+        <v>76.39</v>
       </c>
     </row>
     <row r="10">
@@ -1031,19 +1031,19 @@
         <v>9</v>
       </c>
       <c r="C10" s="10" t="n">
-        <v>9252</v>
+        <v>9200</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>157</v>
+        <v>231</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>2619</v>
+        <v>2597</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>12028</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>76.92</v>
+        <v>76.48999999999999</v>
       </c>
     </row>
     <row r="11">
@@ -1054,19 +1054,19 @@
         <v>10</v>
       </c>
       <c r="C11" s="13" t="n">
-        <v>9163</v>
+        <v>9112</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>159</v>
+        <v>233</v>
       </c>
       <c r="E11" s="13" t="n">
-        <v>2623</v>
+        <v>2600</v>
       </c>
       <c r="F11" s="11" t="n">
         <v>11945</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>76.70999999999999</v>
+        <v>76.28</v>
       </c>
     </row>
     <row r="12">
@@ -1077,19 +1077,19 @@
         <v>11</v>
       </c>
       <c r="C12" s="10" t="n">
-        <v>9121</v>
+        <v>9067</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>157</v>
+        <v>232</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>2620</v>
+        <v>2599</v>
       </c>
       <c r="F12" s="8" t="n">
         <v>11898</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>76.66</v>
+        <v>76.20999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -1100,19 +1100,19 @@
         <v>12</v>
       </c>
       <c r="C13" s="13" t="n">
-        <v>8959</v>
+        <v>8906</v>
       </c>
       <c r="D13" s="11" t="n">
-        <v>156</v>
+        <v>230</v>
       </c>
       <c r="E13" s="13" t="n">
-        <v>2597</v>
+        <v>2576</v>
       </c>
       <c r="F13" s="11" t="n">
         <v>11712</v>
       </c>
       <c r="G13" s="13" t="n">
-        <v>76.48999999999999</v>
+        <v>76.04000000000001</v>
       </c>
     </row>
     <row r="14">
@@ -1123,19 +1123,19 @@
         <v>1</v>
       </c>
       <c r="C14" s="10" t="n">
-        <v>8358</v>
+        <v>8309</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>153</v>
+        <v>222</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>2511</v>
+        <v>2491</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>11022</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>75.83</v>
+        <v>75.39</v>
       </c>
     </row>
     <row r="15">
@@ -1146,19 +1146,19 @@
         <v>2</v>
       </c>
       <c r="C15" s="13" t="n">
-        <v>7583</v>
+        <v>7542</v>
       </c>
       <c r="D15" s="11" t="n">
-        <v>142</v>
+        <v>201</v>
       </c>
       <c r="E15" s="13" t="n">
-        <v>2480</v>
+        <v>2462</v>
       </c>
       <c r="F15" s="11" t="n">
         <v>10205</v>
       </c>
       <c r="G15" s="13" t="n">
-        <v>74.31</v>
+        <v>73.90000000000001</v>
       </c>
     </row>
     <row r="16">
@@ -1169,19 +1169,19 @@
         <v>3</v>
       </c>
       <c r="C16" s="10" t="n">
-        <v>8970</v>
+        <v>8918</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>163</v>
+        <v>236</v>
       </c>
       <c r="E16" s="10" t="n">
-        <v>2625</v>
+        <v>2604</v>
       </c>
       <c r="F16" s="8" t="n">
         <v>11758</v>
       </c>
       <c r="G16" s="10" t="n">
-        <v>76.29000000000001</v>
+        <v>75.84999999999999</v>
       </c>
     </row>
     <row r="17">
@@ -1192,19 +1192,19 @@
         <v>4</v>
       </c>
       <c r="C17" s="13" t="n">
-        <v>9568</v>
+        <v>9513</v>
       </c>
       <c r="D17" s="11" t="n">
-        <v>167</v>
+        <v>243</v>
       </c>
       <c r="E17" s="13" t="n">
-        <v>2681</v>
+        <v>2660</v>
       </c>
       <c r="F17" s="11" t="n">
         <v>12416</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>77.06</v>
+        <v>76.62</v>
       </c>
     </row>
     <row r="18">
@@ -1215,19 +1215,19 @@
         <v>5</v>
       </c>
       <c r="C18" s="10" t="n">
-        <v>9570</v>
+        <v>9513</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>169</v>
+        <v>246</v>
       </c>
       <c r="E18" s="10" t="n">
-        <v>2719</v>
+        <v>2699</v>
       </c>
       <c r="F18" s="8" t="n">
         <v>12458</v>
       </c>
       <c r="G18" s="10" t="n">
-        <v>76.81999999999999</v>
+        <v>76.36</v>
       </c>
     </row>
     <row r="19">
@@ -1238,19 +1238,19 @@
         <v>6</v>
       </c>
       <c r="C19" s="13" t="n">
-        <v>9774</v>
+        <v>9714</v>
       </c>
       <c r="D19" s="11" t="n">
-        <v>165</v>
+        <v>245</v>
       </c>
       <c r="E19" s="13" t="n">
-        <v>2766</v>
+        <v>2746</v>
       </c>
       <c r="F19" s="11" t="n">
         <v>12705</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>76.93000000000001</v>
+        <v>76.45999999999999</v>
       </c>
     </row>
     <row r="20">
@@ -1261,19 +1261,19 @@
         <v>7</v>
       </c>
       <c r="C20" s="10" t="n">
-        <v>9627</v>
+        <v>9570</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>165</v>
+        <v>241</v>
       </c>
       <c r="E20" s="10" t="n">
-        <v>2748</v>
+        <v>2729</v>
       </c>
       <c r="F20" s="8" t="n">
         <v>12540</v>
       </c>
       <c r="G20" s="10" t="n">
-        <v>76.77</v>
+        <v>76.31999999999999</v>
       </c>
     </row>
     <row r="21">
@@ -1284,19 +1284,19 @@
         <v>8</v>
       </c>
       <c r="C21" s="13" t="n">
-        <v>9525</v>
+        <v>9472</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>164</v>
+        <v>237</v>
       </c>
       <c r="E21" s="13" t="n">
-        <v>2759</v>
+        <v>2739</v>
       </c>
       <c r="F21" s="11" t="n">
         <v>12448</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>76.52</v>
+        <v>76.09</v>
       </c>
     </row>
     <row r="22">
@@ -1307,19 +1307,19 @@
         <v>9</v>
       </c>
       <c r="C22" s="10" t="n">
-        <v>9735</v>
+        <v>9678</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>166</v>
+        <v>242</v>
       </c>
       <c r="E22" s="10" t="n">
-        <v>2766</v>
+        <v>2747</v>
       </c>
       <c r="F22" s="8" t="n">
         <v>12667</v>
       </c>
       <c r="G22" s="10" t="n">
-        <v>76.84999999999999</v>
+        <v>76.40000000000001</v>
       </c>
     </row>
     <row r="23">
@@ -1330,19 +1330,19 @@
         <v>10</v>
       </c>
       <c r="C23" s="13" t="n">
-        <v>9710</v>
+        <v>9654</v>
       </c>
       <c r="D23" s="11" t="n">
-        <v>169</v>
+        <v>244</v>
       </c>
       <c r="E23" s="13" t="n">
-        <v>2750</v>
+        <v>2731</v>
       </c>
       <c r="F23" s="11" t="n">
         <v>12629</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>76.89</v>
+        <v>76.44</v>
       </c>
     </row>
     <row r="24">
@@ -1353,19 +1353,19 @@
         <v>11</v>
       </c>
       <c r="C24" s="10" t="n">
-        <v>9746</v>
+        <v>9690</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>170</v>
+        <v>245</v>
       </c>
       <c r="E24" s="10" t="n">
-        <v>2769</v>
+        <v>2750</v>
       </c>
       <c r="F24" s="8" t="n">
         <v>12685</v>
       </c>
       <c r="G24" s="10" t="n">
-        <v>76.83</v>
+        <v>76.39</v>
       </c>
     </row>
     <row r="25">
@@ -1376,19 +1376,19 @@
         <v>12</v>
       </c>
       <c r="C25" s="13" t="n">
-        <v>9688</v>
+        <v>9634</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>168</v>
+        <v>241</v>
       </c>
       <c r="E25" s="13" t="n">
-        <v>2735</v>
+        <v>2716</v>
       </c>
       <c r="F25" s="11" t="n">
         <v>12591</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>76.94</v>
+        <v>76.51000000000001</v>
       </c>
     </row>
     <row r="26">
@@ -1399,19 +1399,19 @@
         <v>1</v>
       </c>
       <c r="C26" s="10" t="n">
-        <v>9049</v>
+        <v>8997</v>
       </c>
       <c r="D26" s="8" t="n">
-        <v>159</v>
+        <v>229</v>
       </c>
       <c r="E26" s="10" t="n">
-        <v>2665</v>
+        <v>2647</v>
       </c>
       <c r="F26" s="8" t="n">
         <v>11873</v>
       </c>
       <c r="G26" s="10" t="n">
-        <v>76.20999999999999</v>
+        <v>75.78</v>
       </c>
     </row>
     <row r="27">
@@ -1422,19 +1422,19 @@
         <v>2</v>
       </c>
       <c r="C27" s="13" t="n">
-        <v>8185</v>
+        <v>8140</v>
       </c>
       <c r="D27" s="11" t="n">
-        <v>145</v>
+        <v>207</v>
       </c>
       <c r="E27" s="13" t="n">
-        <v>2647</v>
+        <v>2630</v>
       </c>
       <c r="F27" s="11" t="n">
         <v>10977</v>
       </c>
       <c r="G27" s="13" t="n">
-        <v>74.56</v>
+        <v>74.16</v>
       </c>
     </row>
     <row r="28">
@@ -1445,19 +1445,19 @@
         <v>3</v>
       </c>
       <c r="C28" s="10" t="n">
-        <v>9437</v>
+        <v>9384</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>158</v>
+        <v>228</v>
       </c>
       <c r="E28" s="10" t="n">
-        <v>2762</v>
+        <v>2745</v>
       </c>
       <c r="F28" s="8" t="n">
         <v>12357</v>
       </c>
       <c r="G28" s="10" t="n">
-        <v>76.37</v>
+        <v>75.94</v>
       </c>
     </row>
     <row r="29">
@@ -1468,19 +1468,19 @@
         <v>4</v>
       </c>
       <c r="C29" s="13" t="n">
-        <v>9981</v>
+        <v>9920</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>170</v>
+        <v>249</v>
       </c>
       <c r="E29" s="13" t="n">
-        <v>2859</v>
+        <v>2841</v>
       </c>
       <c r="F29" s="11" t="n">
         <v>13010</v>
       </c>
       <c r="G29" s="13" t="n">
-        <v>76.72</v>
+        <v>76.25</v>
       </c>
     </row>
     <row r="30">
@@ -1491,19 +1491,19 @@
         <v>5</v>
       </c>
       <c r="C30" s="10" t="n">
-        <v>10140</v>
+        <v>10081</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>169</v>
+        <v>248</v>
       </c>
       <c r="E30" s="10" t="n">
-        <v>2807</v>
+        <v>2787</v>
       </c>
       <c r="F30" s="8" t="n">
         <v>13116</v>
       </c>
       <c r="G30" s="10" t="n">
-        <v>77.31</v>
+        <v>76.86</v>
       </c>
     </row>
     <row r="31">
@@ -1514,19 +1514,19 @@
         <v>6</v>
       </c>
       <c r="C31" s="13" t="n">
-        <v>10163</v>
+        <v>10105</v>
       </c>
       <c r="D31" s="11" t="n">
-        <v>176</v>
+        <v>255</v>
       </c>
       <c r="E31" s="13" t="n">
-        <v>2801</v>
+        <v>2780</v>
       </c>
       <c r="F31" s="11" t="n">
         <v>13140</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>77.34</v>
+        <v>76.90000000000001</v>
       </c>
     </row>
     <row r="32">
@@ -1537,19 +1537,19 @@
         <v>7</v>
       </c>
       <c r="C32" s="10" t="n">
-        <v>10182</v>
+        <v>10127</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>172</v>
+        <v>247</v>
       </c>
       <c r="E32" s="10" t="n">
-        <v>2792</v>
+        <v>2772</v>
       </c>
       <c r="F32" s="8" t="n">
         <v>13146</v>
       </c>
       <c r="G32" s="10" t="n">
-        <v>77.45</v>
+        <v>77.03</v>
       </c>
     </row>
     <row r="33">
@@ -1560,19 +1560,19 @@
         <v>8</v>
       </c>
       <c r="C33" s="13" t="n">
-        <v>9820</v>
+        <v>9768</v>
       </c>
       <c r="D33" s="11" t="n">
-        <v>170</v>
+        <v>241</v>
       </c>
       <c r="E33" s="13" t="n">
-        <v>2786</v>
+        <v>2767</v>
       </c>
       <c r="F33" s="11" t="n">
         <v>12776</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>76.86</v>
+        <v>76.45999999999999</v>
       </c>
     </row>
     <row r="34">
@@ -1583,19 +1583,19 @@
         <v>9</v>
       </c>
       <c r="C34" s="10" t="n">
-        <v>10246</v>
+        <v>10193</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>171</v>
+        <v>244</v>
       </c>
       <c r="E34" s="10" t="n">
-        <v>2792</v>
+        <v>2772</v>
       </c>
       <c r="F34" s="8" t="n">
         <v>13209</v>
       </c>
       <c r="G34" s="10" t="n">
-        <v>77.56999999999999</v>
+        <v>77.17</v>
       </c>
     </row>
     <row r="35">
@@ -1606,19 +1606,19 @@
         <v>10</v>
       </c>
       <c r="C35" s="13" t="n">
-        <v>10317</v>
+        <v>10264</v>
       </c>
       <c r="D35" s="11" t="n">
-        <v>172</v>
+        <v>243</v>
       </c>
       <c r="E35" s="13" t="n">
-        <v>2799</v>
+        <v>2781</v>
       </c>
       <c r="F35" s="11" t="n">
         <v>13288</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>77.64</v>
+        <v>77.23999999999999</v>
       </c>
     </row>
     <row r="36">
@@ -1629,19 +1629,19 @@
         <v>11</v>
       </c>
       <c r="C36" s="10" t="n">
-        <v>10191</v>
+        <v>10138</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>171</v>
+        <v>243</v>
       </c>
       <c r="E36" s="10" t="n">
-        <v>2795</v>
+        <v>2776</v>
       </c>
       <c r="F36" s="8" t="n">
         <v>13157</v>
       </c>
       <c r="G36" s="10" t="n">
-        <v>77.45999999999999</v>
+        <v>77.05</v>
       </c>
     </row>
     <row r="37">
@@ -1652,19 +1652,19 @@
         <v>12</v>
       </c>
       <c r="C37" s="13" t="n">
-        <v>10098</v>
+        <v>10048</v>
       </c>
       <c r="D37" s="11" t="n">
-        <v>170</v>
+        <v>239</v>
       </c>
       <c r="E37" s="13" t="n">
-        <v>2783</v>
+        <v>2764</v>
       </c>
       <c r="F37" s="11" t="n">
         <v>13051</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>77.37</v>
+        <v>76.98999999999999</v>
       </c>
     </row>
     <row r="38">
@@ -1675,19 +1675,19 @@
         <v>1</v>
       </c>
       <c r="C38" s="10" t="n">
-        <v>9584</v>
+        <v>9537</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>167</v>
+        <v>233</v>
       </c>
       <c r="E38" s="10" t="n">
-        <v>2731</v>
+        <v>2712</v>
       </c>
       <c r="F38" s="8" t="n">
         <v>12482</v>
       </c>
       <c r="G38" s="10" t="n">
-        <v>76.78</v>
+        <v>76.41</v>
       </c>
     </row>
     <row r="39">
@@ -1698,19 +1698,19 @@
         <v>2</v>
       </c>
       <c r="C39" s="13" t="n">
-        <v>8200</v>
+        <v>8158</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>152</v>
+        <v>210</v>
       </c>
       <c r="E39" s="13" t="n">
-        <v>2718</v>
+        <v>2702</v>
       </c>
       <c r="F39" s="11" t="n">
         <v>11070</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>74.06999999999999</v>
+        <v>73.69</v>
       </c>
     </row>
     <row r="40">
@@ -1721,19 +1721,19 @@
         <v>3</v>
       </c>
       <c r="C40" s="10" t="n">
-        <v>10348</v>
+        <v>10295</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>178</v>
+        <v>253</v>
       </c>
       <c r="E40" s="10" t="n">
-        <v>2894</v>
+        <v>2872</v>
       </c>
       <c r="F40" s="8" t="n">
         <v>13420</v>
       </c>
       <c r="G40" s="10" t="n">
-        <v>77.11</v>
+        <v>76.70999999999999</v>
       </c>
     </row>
     <row r="41">
@@ -1744,19 +1744,19 @@
         <v>4</v>
       </c>
       <c r="C41" s="13" t="n">
-        <v>10011</v>
+        <v>9961</v>
       </c>
       <c r="D41" s="11" t="n">
-        <v>176</v>
+        <v>244</v>
       </c>
       <c r="E41" s="13" t="n">
-        <v>2861</v>
+        <v>2843</v>
       </c>
       <c r="F41" s="11" t="n">
         <v>13048</v>
       </c>
       <c r="G41" s="13" t="n">
-        <v>76.72</v>
+        <v>76.34</v>
       </c>
     </row>
     <row r="42">
@@ -1767,19 +1767,19 @@
         <v>5</v>
       </c>
       <c r="C42" s="10" t="n">
-        <v>10151</v>
+        <v>10099</v>
       </c>
       <c r="D42" s="8" t="n">
-        <v>180</v>
+        <v>251</v>
       </c>
       <c r="E42" s="10" t="n">
-        <v>2920</v>
+        <v>2901</v>
       </c>
       <c r="F42" s="8" t="n">
         <v>13251</v>
       </c>
       <c r="G42" s="10" t="n">
-        <v>76.61</v>
+        <v>76.20999999999999</v>
       </c>
     </row>
     <row r="43">
@@ -1790,19 +1790,19 @@
         <v>6</v>
       </c>
       <c r="C43" s="13" t="n">
-        <v>10274</v>
+        <v>10223</v>
       </c>
       <c r="D43" s="11" t="n">
-        <v>180</v>
+        <v>250</v>
       </c>
       <c r="E43" s="13" t="n">
-        <v>2917</v>
+        <v>2898</v>
       </c>
       <c r="F43" s="11" t="n">
         <v>13371</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>76.84</v>
+        <v>76.45999999999999</v>
       </c>
     </row>
     <row r="44">
@@ -1813,19 +1813,19 @@
         <v>7</v>
       </c>
       <c r="C44" s="10" t="n">
-        <v>10270</v>
+        <v>10220</v>
       </c>
       <c r="D44" s="8" t="n">
-        <v>181</v>
+        <v>251</v>
       </c>
       <c r="E44" s="10" t="n">
-        <v>2954</v>
+        <v>2934</v>
       </c>
       <c r="F44" s="8" t="n">
         <v>13405</v>
       </c>
       <c r="G44" s="10" t="n">
-        <v>76.61</v>
+        <v>76.23999999999999</v>
       </c>
     </row>
     <row r="45">
@@ -1836,19 +1836,19 @@
         <v>8</v>
       </c>
       <c r="C45" s="13" t="n">
-        <v>9957</v>
+        <v>9908</v>
       </c>
       <c r="D45" s="11" t="n">
-        <v>173</v>
+        <v>242</v>
       </c>
       <c r="E45" s="13" t="n">
-        <v>2932</v>
+        <v>2912</v>
       </c>
       <c r="F45" s="11" t="n">
         <v>13062</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>76.23</v>
+        <v>75.84999999999999</v>
       </c>
     </row>
     <row r="46">
@@ -1859,19 +1859,19 @@
         <v>9</v>
       </c>
       <c r="C46" s="10" t="n">
-        <v>10417</v>
+        <v>10367</v>
       </c>
       <c r="D46" s="8" t="n">
-        <v>175</v>
+        <v>246</v>
       </c>
       <c r="E46" s="10" t="n">
-        <v>2948</v>
+        <v>2927</v>
       </c>
       <c r="F46" s="8" t="n">
         <v>13540</v>
       </c>
       <c r="G46" s="10" t="n">
-        <v>76.94</v>
+        <v>76.56999999999999</v>
       </c>
     </row>
     <row r="47">
@@ -1882,19 +1882,19 @@
         <v>10</v>
       </c>
       <c r="C47" s="13" t="n">
-        <v>10525</v>
+        <v>10473</v>
       </c>
       <c r="D47" s="11" t="n">
-        <v>175</v>
+        <v>250</v>
       </c>
       <c r="E47" s="13" t="n">
-        <v>2954</v>
+        <v>2931</v>
       </c>
       <c r="F47" s="11" t="n">
         <v>13654</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>77.08</v>
+        <v>76.7</v>
       </c>
     </row>
     <row r="48">
@@ -1905,19 +1905,19 @@
         <v>11</v>
       </c>
       <c r="C48" s="10" t="n">
-        <v>10435</v>
+        <v>10384</v>
       </c>
       <c r="D48" s="8" t="n">
-        <v>172</v>
+        <v>246</v>
       </c>
       <c r="E48" s="10" t="n">
-        <v>2939</v>
+        <v>2916</v>
       </c>
       <c r="F48" s="8" t="n">
         <v>13546</v>
       </c>
       <c r="G48" s="10" t="n">
-        <v>77.03</v>
+        <v>76.66</v>
       </c>
     </row>
     <row r="49">
@@ -1928,19 +1928,19 @@
         <v>12</v>
       </c>
       <c r="C49" s="13" t="n">
-        <v>10375</v>
+        <v>10324</v>
       </c>
       <c r="D49" s="11" t="n">
-        <v>170</v>
+        <v>243</v>
       </c>
       <c r="E49" s="13" t="n">
-        <v>2929</v>
+        <v>2907</v>
       </c>
       <c r="F49" s="11" t="n">
         <v>13474</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>77</v>
+        <v>76.62</v>
       </c>
     </row>
     <row r="50">
@@ -1951,19 +1951,19 @@
         <v>1</v>
       </c>
       <c r="C50" s="10" t="n">
-        <v>9887</v>
+        <v>9839</v>
       </c>
       <c r="D50" s="8" t="n">
-        <v>164</v>
+        <v>233</v>
       </c>
       <c r="E50" s="10" t="n">
-        <v>2877</v>
+        <v>2856</v>
       </c>
       <c r="F50" s="8" t="n">
         <v>12928</v>
       </c>
       <c r="G50" s="10" t="n">
-        <v>76.48</v>
+        <v>76.11</v>
       </c>
     </row>
     <row r="51">
@@ -1974,19 +1974,19 @@
         <v>2</v>
       </c>
       <c r="C51" s="13" t="n">
-        <v>7988</v>
+        <v>7948</v>
       </c>
       <c r="D51" s="11" t="n">
-        <v>143</v>
+        <v>200</v>
       </c>
       <c r="E51" s="13" t="n">
-        <v>2769</v>
+        <v>2752</v>
       </c>
       <c r="F51" s="11" t="n">
         <v>10900</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>73.28</v>
+        <v>72.92</v>
       </c>
     </row>
     <row r="52">
@@ -1997,19 +1997,19 @@
         <v>3</v>
       </c>
       <c r="C52" s="10" t="n">
-        <v>10503</v>
+        <v>10451</v>
       </c>
       <c r="D52" s="8" t="n">
-        <v>168</v>
+        <v>243</v>
       </c>
       <c r="E52" s="10" t="n">
-        <v>2897</v>
+        <v>2874</v>
       </c>
       <c r="F52" s="8" t="n">
         <v>13568</v>
       </c>
       <c r="G52" s="10" t="n">
-        <v>77.41</v>
+        <v>77.03</v>
       </c>
     </row>
     <row r="53">
@@ -2020,19 +2020,19 @@
         <v>4</v>
       </c>
       <c r="C53" s="13" t="n">
-        <v>10568</v>
+        <v>10516</v>
       </c>
       <c r="D53" s="11" t="n">
-        <v>167</v>
+        <v>240</v>
       </c>
       <c r="E53" s="13" t="n">
-        <v>2925</v>
+        <v>2904</v>
       </c>
       <c r="F53" s="11" t="n">
         <v>13660</v>
       </c>
       <c r="G53" s="13" t="n">
-        <v>77.36</v>
+        <v>76.98</v>
       </c>
     </row>
     <row r="54">
@@ -2043,19 +2043,19 @@
         <v>5</v>
       </c>
       <c r="C54" s="10" t="n">
-        <v>10454</v>
+        <v>10401</v>
       </c>
       <c r="D54" s="8" t="n">
-        <v>170</v>
+        <v>246</v>
       </c>
       <c r="E54" s="10" t="n">
-        <v>2944</v>
+        <v>2921</v>
       </c>
       <c r="F54" s="8" t="n">
         <v>13568</v>
       </c>
       <c r="G54" s="10" t="n">
-        <v>77.05</v>
+        <v>76.66</v>
       </c>
     </row>
     <row r="55">
@@ -2066,19 +2066,19 @@
         <v>6</v>
       </c>
       <c r="C55" s="13" t="n">
-        <v>10626</v>
+        <v>10571</v>
       </c>
       <c r="D55" s="11" t="n">
-        <v>168</v>
+        <v>247</v>
       </c>
       <c r="E55" s="13" t="n">
-        <v>3057</v>
+        <v>3033</v>
       </c>
       <c r="F55" s="11" t="n">
         <v>13851</v>
       </c>
       <c r="G55" s="13" t="n">
-        <v>76.72</v>
+        <v>76.31999999999999</v>
       </c>
     </row>
     <row r="56">
@@ -2089,19 +2089,19 @@
         <v>7</v>
       </c>
       <c r="C56" s="10" t="n">
-        <v>10656</v>
+        <v>10602</v>
       </c>
       <c r="D56" s="8" t="n">
-        <v>167</v>
+        <v>244</v>
       </c>
       <c r="E56" s="10" t="n">
-        <v>3075</v>
+        <v>3052</v>
       </c>
       <c r="F56" s="8" t="n">
         <v>13898</v>
       </c>
       <c r="G56" s="10" t="n">
-        <v>76.67</v>
+        <v>76.28</v>
       </c>
     </row>
     <row r="57">
@@ -2112,19 +2112,19 @@
         <v>8</v>
       </c>
       <c r="C57" s="13" t="n">
-        <v>10684</v>
+        <v>10631</v>
       </c>
       <c r="D57" s="11" t="n">
-        <v>162</v>
+        <v>239</v>
       </c>
       <c r="E57" s="13" t="n">
-        <v>3070</v>
+        <v>3046</v>
       </c>
       <c r="F57" s="11" t="n">
         <v>13916</v>
       </c>
       <c r="G57" s="13" t="n">
-        <v>76.77</v>
+        <v>76.39</v>
       </c>
     </row>
     <row r="58">
@@ -2135,19 +2135,19 @@
         <v>9</v>
       </c>
       <c r="C58" s="10" t="n">
-        <v>11182</v>
+        <v>11130</v>
       </c>
       <c r="D58" s="8" t="n">
-        <v>172</v>
+        <v>248</v>
       </c>
       <c r="E58" s="10" t="n">
-        <v>3115</v>
+        <v>3091</v>
       </c>
       <c r="F58" s="8" t="n">
         <v>14469</v>
       </c>
       <c r="G58" s="10" t="n">
-        <v>77.28</v>
+        <v>76.92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>